<commit_message>
conditional highlighting not working with new test data
</commit_message>
<xml_diff>
--- a/transportation_safety_report.xlsx
+++ b/transportation_safety_report.xlsx
@@ -468,14 +468,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -486,22 +484,12 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>35 mph</t>
+          <t>25 mph</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>40 mph</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>55 mph</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>70 mph</t>
+          <t>65 mph</t>
         </is>
       </c>
     </row>
@@ -512,16 +500,10 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -531,16 +513,23 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Snow</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3" t="n">
         <v>0</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -554,13 +543,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -588,69 +577,37 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>35 mph</t>
+          <t>25 mph</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>25000</v>
+        <v>12000</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>0.4</v>
+        <v>8.333333333333334</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>40 mph</t>
+          <t>65 mph</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>50000</v>
+        <v>95000</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>55 mph</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>0.1538461538461538</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>70 mph</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>110000</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.3157894736842105</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D5">
+  <conditionalFormatting sqref="D2:D3">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0" stopIfTrue="1">
       <formula>"5"</formula>
     </cfRule>

</xml_diff>

<commit_message>
parse without any corruption popups
</commit_message>
<xml_diff>
--- a/transportation_safety_report.xlsx
+++ b/transportation_safety_report.xlsx
@@ -94,10 +94,8 @@
   <dxfs count="1">
     <dxf>
       <font>
-        <name val="Arial"/>
         <b val="1"/>
         <color rgb="009C0006"/>
-        <sz val="10"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -609,7 +607,7 @@
   </sheetData>
   <conditionalFormatting sqref="D2:D3">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0" stopIfTrue="1">
-      <formula>"5"</formula>
+      <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add a second conditional rule to highlight safe zero-crash zones in green.
</commit_message>
<xml_diff>
--- a/transportation_safety_report.xlsx
+++ b/transportation_safety_report.xlsx
@@ -91,7 +91,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
     <dxf>
       <font>
         <b val="1"/>
@@ -101,6 +101,18 @@
         <patternFill patternType="solid">
           <fgColor rgb="00FFC7CE"/>
           <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+          <bgColor rgb="00C6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -541,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -604,10 +616,79 @@
         <v>0.3157894736842105</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>35 mph</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>45 mph</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>55 mph</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>65000</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>70 mph</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>110000</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D3">
+  <conditionalFormatting sqref="D2:D7">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0" stopIfTrue="1">
       <formula>5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:B7">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1" stopIfTrue="1">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>